<commit_message>
Model v3: Cover target price links to the Valuation FY27 bridge ($120.04, -20.7%)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ArMza8VfAKfU7hr3gFBBh8
</commit_message>
<xml_diff>
--- a/model/Caimanes_Citadel_ABNB_Model_v3.xlsx
+++ b/model/Caimanes_Citadel_ABNB_Model_v3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\krish\citadel-abnb\model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F609B7D-9B78-465B-8FBF-37E0B3DBEF01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C37B45B-CE9C-4FE1-ABC6-15CDA4106471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5360,7 +5360,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1C745F8-7E7E-41C2-B673-61CF08620DAF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23CFE070-3D52-4A48-A767-5FFBE54ADB43}">
   <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -5678,8 +5678,8 @@
     </row>
     <row r="2" spans="1:16" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A2" s="62" t="str">
-        <f>"Target Price: $" &amp; ROUND(AVERAGE(E32:E34),3)</f>
-        <v>Target Price: $120.889</v>
+        <f>"Target Price: $" &amp; ROUND(Valuation!C20,2)</f>
+        <v>Target Price: $120.04</v>
       </c>
       <c r="B2" s="32"/>
       <c r="C2" s="32"/>
@@ -5703,7 +5703,7 @@
     <row r="3" spans="1:16" ht="19.8" x14ac:dyDescent="0.3">
       <c r="A3" s="34" t="str">
         <f>"Target Downside: " &amp; ROUND(E36*100,2) &amp; "%"</f>
-        <v>Target Downside: -20.61%</v>
+        <v>Target Downside: -20.71%</v>
       </c>
       <c r="B3" s="32"/>
       <c r="C3" s="32"/>
@@ -6936,14 +6936,14 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E35" s="3">
-        <f>AVERAGE(E32:E34)-0.7</f>
-        <v>120.18864076954546</v>
+        <f>Valuation!C20</f>
+        <v>120.04219768094279</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E36" s="4">
         <f>E35/P2-1</f>
-        <v>-0.20609920886752453</v>
+        <v>-0.20706653226142546</v>
       </c>
     </row>
   </sheetData>

</xml_diff>